<commit_message>
Add 25-Class Master STEM Curriculum and integrate Mechatron Robotics into catalogue database
</commit_message>
<xml_diff>
--- a/Vendor Research/GoodSoil_Master_Procurement_Database_v1.xlsx
+++ b/Vendor Research/GoodSoil_Master_Procurement_Database_v1.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:O15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="16.7109375" customWidth="1" min="1" max="1"/>
@@ -1455,6 +1455,83 @@
       <c r="N14" t="inlineStr">
         <is>
           <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Mechatron Robotics</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>https://www.mechatronrobotics.com/shop</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Ecosystem</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>4-17</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Robotics, AI, IoT, Electronics, Drones</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>9.5/10</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Reviewed</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>STEM.org Accredited - 12 Store Kits</t>
         </is>
       </c>
     </row>

</xml_diff>